<commit_message>
Drop the rooftop venue: it belonged to another project
The farewell dinner is back at Four Seasons Cairo at Nile Plaza, in a
private area of the hotel, 250 a head with live music - as it was before.
In variant B it stays on board in Aswan on the 29th and the Cairo evening on
the 30th is free again.

The deck keeps its farewell-dinner page, rewritten around the hotel: the
argument there is that nobody travels after dinner, since the rooms are
upstairs. Prices are unchanged - the 250 was the same either way.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KQFm1d6HbwvN6nT4uerjN3
</commit_message>
<xml_diff>
--- a/egypt-jan-2027/Смета_Египет_2027.xlsx
+++ b/egypt-jan-2027/Смета_Египет_2027.xlsx
@@ -987,7 +987,7 @@
     <row r="23">
       <c r="A23" s="11" t="inlineStr">
         <is>
-          <t>Финальный ужин, MOOD Rooftop Cairo</t>
+          <t>Прощальный ужин в Four Seasons</t>
         </is>
       </c>
       <c r="B23" s="6" t="n">
@@ -1008,14 +1008,14 @@
       </c>
       <c r="F23" s="7" t="inlineStr">
         <is>
-          <t>Уточняется. Площадка работает с 22:00 — нужен ранний выкуп. Только вариант A</t>
+          <t>Net или ++? С надбавками 319. Только вариант A</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="11" t="inlineStr">
         <is>
-          <t>Ужин в Lucida или руфтоп</t>
+          <t>Ужин в Lucida</t>
         </is>
       </c>
       <c r="B24" s="6" t="n">
@@ -1829,7 +1829,7 @@
       </c>
       <c r="B7" s="11" t="inlineStr">
         <is>
-          <t>Ужин в Four Seasons: 250 — net или ++? Минимальный счёт за приватную зону сверх меню?</t>
+          <t>Прощальный ужин в Four Seasons: 250 — net или ++? Минимальный счёт за приватную зону?</t>
         </is>
       </c>
       <c r="C7" s="11" t="inlineStr">

</xml_diff>

<commit_message>
Price Khufu's and the Philae dinner, and correct the team's meals in B
Khufu's breakfast at 90 a head and the Philae dinner at 150 a head, both
now line items rather than gaps. Total for the group at sixteen guests:
339 093 for variant A and 403 217 for B; per guest 21 193 and 25 201.
The payment stages still sum exactly to the total.

Also corrected: the team's restaurant meals in variant B were counting the
Four Seasons farewell dinner, which in B happens on board where they already
eat. Their cost there drops accordingly.

Four lines remain without a price: the ground programme for 22-25 January,
Abu Simbel tickets and coach on the ground, airport meet-and-greet, and the
contingency reserve.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KQFm1d6HbwvN6nT4uerjN3
</commit_message>
<xml_diff>
--- a/egypt-jan-2027/Смета_Египет_2027.xlsx
+++ b/egypt-jan-2027/Смета_Египет_2027.xlsx
@@ -550,7 +550,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F42"/>
+  <dimension ref="A1:F43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
@@ -830,119 +830,119 @@
         </is>
       </c>
       <c r="B17" s="6" t="n">
-        <v>0</v>
+        <v>150</v>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>за группу</t>
+          <t>на гостя</t>
         </is>
       </c>
       <c r="D17" s="12">
-        <f>B17/$B$6</f>
+        <f>B17</f>
         <v/>
       </c>
       <c r="E17" s="12">
-        <f>B17/$B$6</f>
-        <v/>
-      </c>
-      <c r="F17" s="8" t="inlineStr">
-        <is>
-          <t>ЦЕНЫ НЕТ. Плюсом к 15 000 EUR</t>
+        <f>B17</f>
+        <v/>
+      </c>
+      <c r="F17" s="7" t="inlineStr">
+        <is>
+          <t>Названо клиентом. Сверх 15 000 EUR за приватный вечер</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="11" t="inlineStr">
         <is>
-          <t>Гиза: приватный доступ, одно посещение</t>
+          <t>Завтрак в Khufu’s</t>
         </is>
       </c>
       <c r="B18" s="6" t="n">
-        <v>3500</v>
+        <v>90</v>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>за посещение</t>
+          <t>на гостя</t>
         </is>
       </c>
       <c r="D18" s="12">
-        <f>B18*2/$B$6</f>
+        <f>B18</f>
         <v/>
       </c>
       <c r="E18" s="12">
-        <f>B18*2/$B$6</f>
+        <f>B18</f>
         <v/>
       </c>
       <c r="F18" s="7" t="inlineStr">
         <is>
-          <t>ПОДТВЕРЖДЕНО: персональное разрешение, доступ во все зоны. Нужно два</t>
+          <t>Названо клиентом</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="11" t="inlineStr">
         <is>
-          <t>Абу-Симбел самолётом</t>
+          <t>Гиза: приватный доступ, одно посещение</t>
         </is>
       </c>
       <c r="B19" s="6" t="n">
-        <v>470</v>
+        <v>3500</v>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>на гостя</t>
+          <t>за посещение</t>
         </is>
       </c>
       <c r="D19" s="12">
-        <f>B19</f>
+        <f>B19*2/$B$6</f>
         <v/>
       </c>
       <c r="E19" s="12">
-        <f>B19</f>
+        <f>B19*2/$B$6</f>
         <v/>
       </c>
       <c r="F19" s="7" t="inlineStr">
         <is>
-          <t>Обязательная часть для всех. Альтернатива по земле — см. лист «Абу-Симбел»</t>
+          <t>ПОДТВЕРЖДЕНО: персональное разрешение, доступ во все зоны. Нужно два</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="11" t="inlineStr">
         <is>
-          <t>Giza Palace, ночь</t>
+          <t>Абу-Симбел самолётом</t>
         </is>
       </c>
       <c r="B20" s="6" t="n">
-        <v>325</v>
+        <v>470</v>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>за номер за ночь</t>
+          <t>на гостя</t>
         </is>
       </c>
       <c r="D20" s="12">
-        <f>B20*2</f>
+        <f>B20</f>
         <v/>
       </c>
       <c r="E20" s="12">
-        <f>B20*2</f>
+        <f>B20</f>
         <v/>
       </c>
       <c r="F20" s="7" t="inlineStr">
         <is>
-          <t>Две ночи. Открытые источники 222–349. Запросить групповой тариф</t>
+          <t>Обязательная часть для всех. Альтернатива по земле — см. лист «Абу-Симбел»</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="11" t="inlineStr">
         <is>
-          <t>Steigenberger Nile Palace, ночь</t>
+          <t>Giza Palace, ночь</t>
         </is>
       </c>
       <c r="B21" s="6" t="n">
-        <v>170</v>
+        <v>325</v>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
@@ -950,31 +950,31 @@
         </is>
       </c>
       <c r="D21" s="12">
-        <f>B21</f>
+        <f>B21*2</f>
         <v/>
       </c>
       <c r="E21" s="12">
-        <f>B21</f>
+        <f>B21*2</f>
         <v/>
       </c>
       <c r="F21" s="7" t="inlineStr">
         <is>
-          <t>Открытые источники 120–176. Запросить групповой тариф</t>
+          <t>Две ночи. Открытые источники 222–349. Запросить групповой тариф</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="11" t="inlineStr">
         <is>
-          <t>Отель 29 января: Асуан (A) / Four Seasons 30-го (B)</t>
+          <t>Steigenberger Nile Palace, ночь</t>
         </is>
       </c>
       <c r="B22" s="6" t="n">
-        <v>250</v>
+        <v>170</v>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>на гостя</t>
+          <t>за номер за ночь</t>
         </is>
       </c>
       <c r="D22" s="12">
@@ -982,19 +982,19 @@
         <v/>
       </c>
       <c r="E22" s="12">
-        <f>570</f>
+        <f>B22</f>
         <v/>
       </c>
       <c r="F22" s="7" t="inlineStr">
         <is>
-          <t>A: остров Элефантина, открытые источники 140–330. B: Four Seasons, 570 названо отелем</t>
+          <t>Открытые источники 120–176. Запросить групповой тариф</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="11" t="inlineStr">
         <is>
-          <t>Прощальный ужин в Four Seasons</t>
+          <t>Отель 29 января: Асуан (A) / Four Seasons 30-го (B)</t>
         </is>
       </c>
       <c r="B23" s="6" t="n">
@@ -1010,23 +1010,23 @@
         <v/>
       </c>
       <c r="E23" s="12">
-        <f>0</f>
+        <f>570</f>
         <v/>
       </c>
       <c r="F23" s="7" t="inlineStr">
         <is>
-          <t>Net или ++? С надбавками 319. Только вариант A</t>
+          <t>A: остров Элефантина, открытые источники 140–330. B: Four Seasons, 570 названо отелем</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="11" t="inlineStr">
         <is>
-          <t>Ужин в Lucida</t>
+          <t>Прощальный ужин в Four Seasons</t>
         </is>
       </c>
       <c r="B24" s="6" t="n">
-        <v>150</v>
+        <v>250</v>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
@@ -1038,23 +1038,23 @@
         <v/>
       </c>
       <c r="E24" s="12">
-        <f>B24</f>
+        <f>0</f>
         <v/>
       </c>
       <c r="F24" s="7" t="inlineStr">
         <is>
-          <t>ПОДТВЕРЖДЕНО: 150 без алкоголя</t>
+          <t>Net или ++? С надбавками 319. Только вариант A</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="11" t="inlineStr">
         <is>
-          <t>Питание в отелях вне названных ресторанов</t>
+          <t>Ужин в Lucida</t>
         </is>
       </c>
       <c r="B25" s="6" t="n">
-        <v>200</v>
+        <v>150</v>
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
@@ -1071,50 +1071,50 @@
       </c>
       <c r="F25" s="7" t="inlineStr">
         <is>
-          <t>Наша оценка на всю поездку: ужин 40–60, обед 25–35</t>
+          <t>ПОДТВЕРЖДЕНО: 150 без алкоголя</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="11" t="inlineStr">
         <is>
-          <t>Полёт на шаре, две корзины</t>
+          <t>Питание в отелях вне названных ресторанов</t>
         </is>
       </c>
       <c r="B26" s="6" t="n">
-        <v>5000</v>
+        <v>200</v>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>за все корзины</t>
+          <t>на гостя</t>
         </is>
       </c>
       <c r="D26" s="12">
-        <f>B26/$B$6</f>
+        <f>B26</f>
         <v/>
       </c>
       <c r="E26" s="12">
-        <f>B26/$B$6</f>
+        <f>B26</f>
         <v/>
       </c>
       <c r="F26" s="7" t="inlineStr">
         <is>
-          <t>ПОДТВЕРЖДЕНО: две корзины, по 8 человек</t>
+          <t>Наша оценка на всю поездку: ужин 40–60, обед 25–35</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="11" t="inlineStr">
         <is>
-          <t>Нубийский ансамбль</t>
+          <t>Полёт на шаре, две корзины</t>
         </is>
       </c>
       <c r="B27" s="6" t="n">
-        <v>650</v>
+        <v>5000</v>
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>за вечер</t>
+          <t>за все корзины</t>
         </is>
       </c>
       <c r="D27" s="12">
@@ -1127,42 +1127,42 @@
       </c>
       <c r="F27" s="7" t="inlineStr">
         <is>
-          <t>Наша оценка 400–900. Публичных прайсов нет</t>
+          <t>ПОДТВЕРЖДЕНО: две корзины, по 8 человек</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="11" t="inlineStr">
         <is>
-          <t>Гала-ужин на борту, вариант B</t>
+          <t>Нубийский ансамбль</t>
         </is>
       </c>
       <c r="B28" s="6" t="n">
-        <v>0</v>
+        <v>650</v>
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>за группу</t>
+          <t>за вечер</t>
         </is>
       </c>
       <c r="D28" s="12">
-        <f>0</f>
+        <f>B28/$B$6</f>
         <v/>
       </c>
       <c r="E28" s="12">
         <f>B28/$B$6</f>
         <v/>
       </c>
-      <c r="F28" s="8" t="inlineStr">
-        <is>
-          <t>ЦЕНЫ НЕТ. Меню, декор, музыка сверх пансиона</t>
+      <c r="F28" s="7" t="inlineStr">
+        <is>
+          <t>Наша оценка 400–900. Публичных прайсов нет</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="11" t="inlineStr">
         <is>
-          <t>Наземная программа 22–25 января</t>
+          <t>Гала-ужин на борту, вариант B</t>
         </is>
       </c>
       <c r="B29" s="6" t="n">
@@ -1174,7 +1174,7 @@
         </is>
       </c>
       <c r="D29" s="12">
-        <f>B29/$B$6</f>
+        <f>0</f>
         <v/>
       </c>
       <c r="E29" s="12">
@@ -1183,46 +1183,46 @@
       </c>
       <c r="F29" s="8" t="inlineStr">
         <is>
-          <t>ЦЕНЫ НЕТ. Гид, транспорт, билеты, GEM. Крупнейшая дыра в смете</t>
+          <t>ЦЕНЫ НЕТ. Меню, декор, музыка сверх пансиона</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="11" t="inlineStr">
         <is>
-          <t>Перелёты Каир–Луксор и Асуан–Каир</t>
+          <t>Наземная программа 22–25 января</t>
         </is>
       </c>
       <c r="B30" s="6" t="n">
-        <v>250</v>
+        <v>0</v>
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>на гостя</t>
+          <t>за группу</t>
         </is>
       </c>
       <c r="D30" s="12">
-        <f>B30</f>
+        <f>B30/$B$6</f>
         <v/>
       </c>
       <c r="E30" s="12">
-        <f>B30</f>
-        <v/>
-      </c>
-      <c r="F30" s="7" t="inlineStr">
-        <is>
-          <t>ОЦЕНКА по открытым источникам: 140 + 110. Групповой тариф запрошен</t>
+        <f>B30/$B$6</f>
+        <v/>
+      </c>
+      <c r="F30" s="8" t="inlineStr">
+        <is>
+          <t>ЦЕНЫ НЕТ. Гид, транспорт, билеты, GEM. Крупнейшая дыра в смете</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="11" t="inlineStr">
         <is>
-          <t>Прочее: Khufu's, meet &amp; greet, fast track</t>
+          <t>Перелёты Каир–Луксор и Асуан–Каир</t>
         </is>
       </c>
       <c r="B31" s="6" t="n">
-        <v>0</v>
+        <v>250</v>
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
@@ -1237,16 +1237,16 @@
         <f>B31</f>
         <v/>
       </c>
-      <c r="F31" s="8" t="inlineStr">
-        <is>
-          <t>ЦЕНЫ НЕТ</t>
+      <c r="F31" s="7" t="inlineStr">
+        <is>
+          <t>ОЦЕНКА по открытым источникам: 140 + 110. Групповой тариф запрошен</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="11" t="inlineStr">
         <is>
-          <t>Резерв на решения на месте</t>
+          <t>Прочее: meet &amp; greet, fast track</t>
         </is>
       </c>
       <c r="B32" s="6" t="n">
@@ -1265,167 +1265,195 @@
         <f>B32</f>
         <v/>
       </c>
-      <c r="F32" s="7" t="inlineStr">
-        <is>
-          <t>НЕ ЗАЛОЖЕН. Обычно 2–3 % от сметы. Ваше решение</t>
+      <c r="F32" s="8" t="inlineStr">
+        <is>
+          <t>ЦЕНЫ НЕТ</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="11" t="inlineStr">
         <is>
-          <t>ПРОПУЩЕННЫЕ СТАТЬИ — итог с листа «Пропущено»</t>
-        </is>
-      </c>
-      <c r="B33" s="12">
-        <f>Пропущено!$B$19</f>
-        <v/>
+          <t>Резерв на решения на месте</t>
+        </is>
+      </c>
+      <c r="B33" s="6" t="n">
+        <v>0</v>
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>за группу</t>
+          <t>на гостя</t>
         </is>
       </c>
       <c r="D33" s="12">
-        <f>B33/$B$6</f>
+        <f>B33</f>
         <v/>
       </c>
       <c r="E33" s="12">
-        <f>B33/$B$6</f>
+        <f>B33</f>
         <v/>
       </c>
       <c r="F33" s="7" t="inlineStr">
         <is>
-          <t>Двенадцать позиций, найденных при сверке. Пока нули</t>
+          <t>НЕ ЗАЛОЖЕН. Обычно 2–3 % от сметы. Ваше решение</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="11" t="inlineStr">
         <is>
+          <t>ПРОПУЩЕННЫЕ СТАТЬИ — итог с листа «Пропущено»</t>
+        </is>
+      </c>
+      <c r="B34" s="12">
+        <f>Пропущено!$B$19</f>
+        <v/>
+      </c>
+      <c r="C34" s="2" t="inlineStr">
+        <is>
+          <t>за группу</t>
+        </is>
+      </c>
+      <c r="D34" s="12">
+        <f>B34/$B$6</f>
+        <v/>
+      </c>
+      <c r="E34" s="12">
+        <f>B34/$B$6</f>
+        <v/>
+      </c>
+      <c r="F34" s="7" t="inlineStr">
+        <is>
+          <t>Двенадцать позиций, найденных при сверке. Пока нули</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="11" t="inlineStr">
+        <is>
           <t>КОМАНДА LA ROYAL</t>
         </is>
       </c>
-      <c r="B34" s="12">
+      <c r="B35" s="12">
         <f>Команда!$B$22</f>
         <v/>
       </c>
-      <c r="C34" s="2" t="inlineStr">
+      <c r="C35" s="2" t="inlineStr">
         <is>
           <t>за группу</t>
         </is>
       </c>
-      <c r="D34" s="12">
-        <f>B34*Команда!$B$24/$B$6</f>
-        <v/>
-      </c>
-      <c r="E34" s="12">
-        <f>B34*Команда!$B$24/$B$6</f>
-        <v/>
-      </c>
-      <c r="F34" s="7" t="inlineStr">
+      <c r="D35" s="12">
+        <f>B35*Команда!$B$24/$B$6</f>
+        <v/>
+      </c>
+      <c r="E35" s="12">
+        <f>B35*Команда!$B$24/$B$6</f>
+        <v/>
+      </c>
+      <c r="F35" s="7" t="inlineStr">
         <is>
           <t>Переключатель «в себестоимость / из вознаграждения» — на листе «Команда»</t>
         </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="5" t="inlineStr">
-        <is>
-          <t>СЕБЕСТОИМОСТЬ НА ГОСТЯ</t>
-        </is>
-      </c>
-      <c r="D35" s="13">
-        <f>SUM(D15:D34)</f>
-        <v/>
-      </c>
-      <c r="E35" s="13">
-        <f>SUM(E15:E34)</f>
-        <v/>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="5" t="inlineStr">
         <is>
+          <t>СЕБЕСТОИМОСТЬ НА ГОСТЯ</t>
+        </is>
+      </c>
+      <c r="D36" s="13">
+        <f>SUM(D15:D35)</f>
+        <v/>
+      </c>
+      <c r="E36" s="13">
+        <f>SUM(E15:E35)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="5" t="inlineStr">
+        <is>
           <t>Вознаграждение La Royal</t>
         </is>
       </c>
-      <c r="D36" s="12">
-        <f>D35*$B$11</f>
-        <v/>
-      </c>
-      <c r="E36" s="12">
-        <f>E35*$B$11</f>
-        <v/>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="14" t="inlineStr">
+      <c r="D37" s="12">
+        <f>D36*$B$11</f>
+        <v/>
+      </c>
+      <c r="E37" s="12">
+        <f>E36*$B$11</f>
+        <v/>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="14" t="inlineStr">
         <is>
           <t>ЦЕНА ДЛЯ ГОСТЯ</t>
         </is>
       </c>
-      <c r="D37" s="15">
-        <f>D35+D36</f>
-        <v/>
-      </c>
-      <c r="E37" s="15">
-        <f>E35+E36</f>
-        <v/>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="2" t="inlineStr">
-        <is>
-          <t>Вознаграждение со всей группы</t>
-        </is>
-      </c>
-      <c r="D38" s="16">
-        <f>D36*$B$6-Команда!$B$22*(1-Команда!$B$24)</f>
-        <v/>
-      </c>
-      <c r="E38" s="16">
-        <f>E36*$B$6-Команда!$B$22*(1-Команда!$B$24)</f>
-        <v/>
-      </c>
-      <c r="F38" s="2" t="inlineStr">
-        <is>
-          <t>Если команда идёт из вознаграждения, её расходы вычитаются здесь</t>
-        </is>
+      <c r="D38" s="15">
+        <f>D36+D37</f>
+        <v/>
+      </c>
+      <c r="E38" s="15">
+        <f>E36+E37</f>
+        <v/>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>Если 15 % считать долей в цене, а не наценкой</t>
-        </is>
-      </c>
-      <c r="D39" s="17">
-        <f>D35/(1-$B$11)</f>
-        <v/>
-      </c>
-      <c r="E39" s="17">
-        <f>E35/(1-$B$11)</f>
-        <v/>
+          <t>Вознаграждение со всей группы</t>
+        </is>
+      </c>
+      <c r="D39" s="16">
+        <f>D37*$B$6-Команда!$B$22*(1-Команда!$B$24)</f>
+        <v/>
+      </c>
+      <c r="E39" s="16">
+        <f>E37*$B$6-Команда!$B$22*(1-Команда!$B$24)</f>
+        <v/>
+      </c>
+      <c r="F39" s="2" t="inlineStr">
+        <is>
+          <t>Если команда идёт из вознаграждения, её расходы вычитаются здесь</t>
+        </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
+          <t>Если 15 % считать долей в цене, а не наценкой</t>
+        </is>
+      </c>
+      <c r="D40" s="17">
+        <f>D36/(1-$B$11)</f>
+        <v/>
+      </c>
+      <c r="E40" s="17">
+        <f>E36/(1-$B$11)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="2" t="inlineStr">
+        <is>
           <t>Разница между двумя трактовками, на гостя</t>
         </is>
       </c>
-      <c r="D40" s="17">
-        <f>D39-D37</f>
-        <v/>
-      </c>
-      <c r="E40" s="17">
-        <f>E39-E37</f>
-        <v/>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" s="18" t="inlineStr">
+      <c r="D41" s="17">
+        <f>D40-D38</f>
+        <v/>
+      </c>
+      <c r="E41" s="17">
+        <f>E40-E38</f>
+        <v/>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="18" t="inlineStr">
         <is>
           <t>Пока в столбце «Что уточнить» есть розовые строки, итог занижен и клиенту не называется.</t>
         </is>
@@ -1689,16 +1717,16 @@
     <row r="19">
       <c r="A19" s="11" t="inlineStr">
         <is>
-          <t>Ужины в Lucida и Four Seasons</t>
+          <t>Ужины вне борта: Lucida, Филе, Khufu, прощальный</t>
         </is>
       </c>
       <c r="B19" s="12">
-        <f>$B$7*400</f>
+        <f>$B$7*640</f>
         <v/>
       </c>
       <c r="D19" s="7" t="inlineStr">
         <is>
-          <t>150 + 250 на человека</t>
+          <t>150+150+90+250 на человека</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Separate the Giza tickets from the private opening
The 3 500 buys the private opening for the group; tickets are on top at 180
a head. Two openings and sixteen guests make 7 000 plus 5 760, plus the
escorts' tickets. Variant A rises to 349 029 for the group, 21 814 a guest;
variant B to 413 153. Both payment halves move with it.

Two questions in the internal file. I have assumed a ticket per person per
visit, morning and night; if one ticket covers both, the estimate drops by
2 880. And what the 180 covers - the public gate is 700 EGP for the plateau
and 1 500 more for the Khufu interior, about 44 dollars all in, so 180 is
the out-of-hours tariff, which is normal, but if the interior is already
inside it then the separate option is unnecessary.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KQFm1d6HbwvN6nT4uerjN3
</commit_message>
<xml_diff>
--- a/egypt-jan-2027/Смета_Египет_2027.xlsx
+++ b/egypt-jan-2027/Смета_Египет_2027.xlsx
@@ -550,7 +550,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F44"/>
+  <dimension ref="A1:F45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
@@ -931,74 +931,74 @@
       </c>
       <c r="F20" s="7" t="inlineStr">
         <is>
-          <t>ПОДТВЕРЖДЕНО: персональное разрешение, доступ во все зоны. Нужно два</t>
+          <t>ПОДТВЕРЖДЕНО: приватное открытие для группы. Билеты НЕ входят, см. строку ниже</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="11" t="inlineStr">
         <is>
-          <t>Абу-Симбел самолётом</t>
+          <t>Входной билет на плато Гизы</t>
         </is>
       </c>
       <c r="B21" s="6" t="n">
-        <v>470</v>
+        <v>180</v>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>на гостя</t>
+          <t>за билет</t>
         </is>
       </c>
       <c r="D21" s="12">
-        <f>B21</f>
+        <f>B21*2</f>
         <v/>
       </c>
       <c r="E21" s="12">
-        <f>B21</f>
-        <v/>
-      </c>
-      <c r="F21" s="7" t="inlineStr">
-        <is>
-          <t>Обязательная часть для всех. Альтернатива по земле — см. лист «Абу-Симбел»</t>
+        <f>B21*2</f>
+        <v/>
+      </c>
+      <c r="F21" s="8" t="inlineStr">
+        <is>
+          <t>180 за билет. ПРОВЕРИТЬ: один билет на оба посещения или два</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="11" t="inlineStr">
         <is>
-          <t>Giza Palace, ночь</t>
+          <t>Абу-Симбел самолётом</t>
         </is>
       </c>
       <c r="B22" s="6" t="n">
-        <v>325</v>
+        <v>470</v>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>за номер за ночь</t>
+          <t>на гостя</t>
         </is>
       </c>
       <c r="D22" s="12">
-        <f>B22*2</f>
+        <f>B22</f>
         <v/>
       </c>
       <c r="E22" s="12">
-        <f>B22*2</f>
+        <f>B22</f>
         <v/>
       </c>
       <c r="F22" s="7" t="inlineStr">
         <is>
-          <t>Две ночи. Открытые источники 222–349. Запросить групповой тариф</t>
+          <t>Обязательная часть для всех. Альтернатива по земле — см. лист «Абу-Симбел»</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="11" t="inlineStr">
         <is>
-          <t>Steigenberger Nile Palace, ночь</t>
+          <t>Giza Palace, ночь</t>
         </is>
       </c>
       <c r="B23" s="6" t="n">
-        <v>170</v>
+        <v>325</v>
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
@@ -1006,31 +1006,31 @@
         </is>
       </c>
       <c r="D23" s="12">
-        <f>B23</f>
+        <f>B23*2</f>
         <v/>
       </c>
       <c r="E23" s="12">
-        <f>B23</f>
+        <f>B23*2</f>
         <v/>
       </c>
       <c r="F23" s="7" t="inlineStr">
         <is>
-          <t>Открытые источники 120–176. Запросить групповой тариф</t>
+          <t>Две ночи. Открытые источники 222–349. Запросить групповой тариф</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="11" t="inlineStr">
         <is>
-          <t>Отель 29 января: Асуан (A) / Four Seasons 30-го (B)</t>
+          <t>Steigenberger Nile Palace, ночь</t>
         </is>
       </c>
       <c r="B24" s="6" t="n">
-        <v>250</v>
+        <v>170</v>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>на гостя</t>
+          <t>за номер за ночь</t>
         </is>
       </c>
       <c r="D24" s="12">
@@ -1038,19 +1038,19 @@
         <v/>
       </c>
       <c r="E24" s="12">
-        <f>570</f>
+        <f>B24</f>
         <v/>
       </c>
       <c r="F24" s="7" t="inlineStr">
         <is>
-          <t>A: остров Элефантина, открытые источники 140–330. B: Four Seasons, 570 названо отелем</t>
+          <t>Открытые источники 120–176. Запросить групповой тариф</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="11" t="inlineStr">
         <is>
-          <t>Прощальный ужин в Four Seasons</t>
+          <t>Отель 29 января: Асуан (A) / Four Seasons 30-го (B)</t>
         </is>
       </c>
       <c r="B25" s="6" t="n">
@@ -1066,23 +1066,23 @@
         <v/>
       </c>
       <c r="E25" s="12">
-        <f>0</f>
+        <f>570</f>
         <v/>
       </c>
       <c r="F25" s="7" t="inlineStr">
         <is>
-          <t>Net или ++? С надбавками 319. Только вариант A</t>
+          <t>A: остров Элефантина, открытые источники 140–330. B: Four Seasons, 570 названо отелем</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="11" t="inlineStr">
         <is>
-          <t>Ужин в Lucida</t>
+          <t>Прощальный ужин в Four Seasons</t>
         </is>
       </c>
       <c r="B26" s="6" t="n">
-        <v>150</v>
+        <v>250</v>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
@@ -1094,23 +1094,23 @@
         <v/>
       </c>
       <c r="E26" s="12">
-        <f>B26</f>
+        <f>0</f>
         <v/>
       </c>
       <c r="F26" s="7" t="inlineStr">
         <is>
-          <t>ПОДТВЕРЖДЕНО: 150 без алкоголя</t>
+          <t>Net или ++? С надбавками 319. Только вариант A</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="11" t="inlineStr">
         <is>
-          <t>Питание в отелях вне названных ресторанов</t>
+          <t>Ужин в Lucida</t>
         </is>
       </c>
       <c r="B27" s="6" t="n">
-        <v>200</v>
+        <v>150</v>
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
@@ -1127,50 +1127,50 @@
       </c>
       <c r="F27" s="7" t="inlineStr">
         <is>
-          <t>Наша оценка на всю поездку: ужин 40–60, обед 25–35</t>
+          <t>ПОДТВЕРЖДЕНО: 150 без алкоголя</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="11" t="inlineStr">
         <is>
-          <t>Полёт на шаре, две корзины</t>
+          <t>Питание в отелях вне названных ресторанов</t>
         </is>
       </c>
       <c r="B28" s="6" t="n">
-        <v>5000</v>
+        <v>200</v>
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>за все корзины</t>
+          <t>на гостя</t>
         </is>
       </c>
       <c r="D28" s="12">
-        <f>B28/$B$6</f>
+        <f>B28</f>
         <v/>
       </c>
       <c r="E28" s="12">
-        <f>B28/$B$6</f>
+        <f>B28</f>
         <v/>
       </c>
       <c r="F28" s="7" t="inlineStr">
         <is>
-          <t>ПОДТВЕРЖДЕНО: две корзины, по 8 человек</t>
+          <t>Наша оценка на всю поездку: ужин 40–60, обед 25–35</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="11" t="inlineStr">
         <is>
-          <t>Нубийский ансамбль</t>
+          <t>Полёт на шаре, две корзины</t>
         </is>
       </c>
       <c r="B29" s="6" t="n">
-        <v>650</v>
+        <v>5000</v>
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>за вечер</t>
+          <t>за все корзины</t>
         </is>
       </c>
       <c r="D29" s="12">
@@ -1183,42 +1183,42 @@
       </c>
       <c r="F29" s="7" t="inlineStr">
         <is>
-          <t>Наша оценка 400–900. Публичных прайсов нет</t>
+          <t>ПОДТВЕРЖДЕНО: две корзины, по 8 человек</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="11" t="inlineStr">
         <is>
-          <t>Гала-ужин на борту, вариант B</t>
+          <t>Нубийский ансамбль</t>
         </is>
       </c>
       <c r="B30" s="6" t="n">
-        <v>0</v>
+        <v>650</v>
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>за группу</t>
+          <t>за вечер</t>
         </is>
       </c>
       <c r="D30" s="12">
-        <f>0</f>
+        <f>B30/$B$6</f>
         <v/>
       </c>
       <c r="E30" s="12">
         <f>B30/$B$6</f>
         <v/>
       </c>
-      <c r="F30" s="8" t="inlineStr">
-        <is>
-          <t>ЦЕНЫ НЕТ. Меню, декор, музыка сверх пансиона</t>
+      <c r="F30" s="7" t="inlineStr">
+        <is>
+          <t>Наша оценка 400–900. Публичных прайсов нет</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="11" t="inlineStr">
         <is>
-          <t>Наземная программа 22–25 января</t>
+          <t>Гала-ужин на борту, вариант B</t>
         </is>
       </c>
       <c r="B31" s="6" t="n">
@@ -1230,7 +1230,7 @@
         </is>
       </c>
       <c r="D31" s="12">
-        <f>B31/$B$6</f>
+        <f>0</f>
         <v/>
       </c>
       <c r="E31" s="12">
@@ -1239,46 +1239,46 @@
       </c>
       <c r="F31" s="8" t="inlineStr">
         <is>
-          <t>ЦЕНЫ НЕТ. Гид, транспорт, билеты, GEM. Крупнейшая дыра в смете</t>
+          <t>ЦЕНЫ НЕТ. Меню, декор, музыка сверх пансиона</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="11" t="inlineStr">
         <is>
-          <t>Перелёты Каир–Луксор и Асуан–Каир</t>
+          <t>Наземная программа 22–25 января</t>
         </is>
       </c>
       <c r="B32" s="6" t="n">
-        <v>250</v>
+        <v>0</v>
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>на гостя</t>
+          <t>за группу</t>
         </is>
       </c>
       <c r="D32" s="12">
-        <f>B32</f>
+        <f>B32/$B$6</f>
         <v/>
       </c>
       <c r="E32" s="12">
-        <f>B32</f>
-        <v/>
-      </c>
-      <c r="F32" s="7" t="inlineStr">
-        <is>
-          <t>ОЦЕНКА по открытым источникам: 140 + 110. Групповой тариф запрошен</t>
+        <f>B32/$B$6</f>
+        <v/>
+      </c>
+      <c r="F32" s="8" t="inlineStr">
+        <is>
+          <t>ЦЕНЫ НЕТ. Гид, транспорт, билеты, GEM. Крупнейшая дыра в смете</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="11" t="inlineStr">
         <is>
-          <t>Прочее: meet &amp; greet, fast track</t>
+          <t>Перелёты Каир–Луксор и Асуан–Каир</t>
         </is>
       </c>
       <c r="B33" s="6" t="n">
-        <v>0</v>
+        <v>250</v>
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
@@ -1293,16 +1293,16 @@
         <f>B33</f>
         <v/>
       </c>
-      <c r="F33" s="8" t="inlineStr">
-        <is>
-          <t>ЦЕНЫ НЕТ</t>
+      <c r="F33" s="7" t="inlineStr">
+        <is>
+          <t>ОЦЕНКА по открытым источникам: 140 + 110. Групповой тариф запрошен</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="11" t="inlineStr">
         <is>
-          <t>Резерв на решения на месте</t>
+          <t>Прочее: meet &amp; greet, fast track</t>
         </is>
       </c>
       <c r="B34" s="6" t="n">
@@ -1321,167 +1321,195 @@
         <f>B34</f>
         <v/>
       </c>
-      <c r="F34" s="7" t="inlineStr">
-        <is>
-          <t>НЕ ЗАЛОЖЕН. Обычно 2–3 % от сметы. Ваше решение</t>
+      <c r="F34" s="8" t="inlineStr">
+        <is>
+          <t>ЦЕНЫ НЕТ</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="11" t="inlineStr">
         <is>
-          <t>ПРОПУЩЕННЫЕ СТАТЬИ — итог с листа «Пропущено»</t>
-        </is>
-      </c>
-      <c r="B35" s="12">
-        <f>Пропущено!$B$19</f>
-        <v/>
+          <t>Резерв на решения на месте</t>
+        </is>
+      </c>
+      <c r="B35" s="6" t="n">
+        <v>0</v>
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>за группу</t>
+          <t>на гостя</t>
         </is>
       </c>
       <c r="D35" s="12">
-        <f>B35/$B$6</f>
+        <f>B35</f>
         <v/>
       </c>
       <c r="E35" s="12">
-        <f>B35/$B$6</f>
+        <f>B35</f>
         <v/>
       </c>
       <c r="F35" s="7" t="inlineStr">
         <is>
-          <t>Двенадцать позиций, найденных при сверке. Пока нули</t>
+          <t>НЕ ЗАЛОЖЕН. Обычно 2–3 % от сметы. Ваше решение</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="11" t="inlineStr">
         <is>
+          <t>ПРОПУЩЕННЫЕ СТАТЬИ — итог с листа «Пропущено»</t>
+        </is>
+      </c>
+      <c r="B36" s="12">
+        <f>Пропущено!$B$19</f>
+        <v/>
+      </c>
+      <c r="C36" s="2" t="inlineStr">
+        <is>
+          <t>за группу</t>
+        </is>
+      </c>
+      <c r="D36" s="12">
+        <f>B36/$B$6</f>
+        <v/>
+      </c>
+      <c r="E36" s="12">
+        <f>B36/$B$6</f>
+        <v/>
+      </c>
+      <c r="F36" s="7" t="inlineStr">
+        <is>
+          <t>Двенадцать позиций, найденных при сверке. Пока нули</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="11" t="inlineStr">
+        <is>
           <t>КОМАНДА LA ROYAL</t>
         </is>
       </c>
-      <c r="B36" s="12">
+      <c r="B37" s="12">
         <f>Команда!$B$22</f>
         <v/>
       </c>
-      <c r="C36" s="2" t="inlineStr">
+      <c r="C37" s="2" t="inlineStr">
         <is>
           <t>за группу</t>
         </is>
       </c>
-      <c r="D36" s="12">
-        <f>B36*Команда!$B$24/$B$6</f>
-        <v/>
-      </c>
-      <c r="E36" s="12">
-        <f>B36*Команда!$B$24/$B$6</f>
-        <v/>
-      </c>
-      <c r="F36" s="7" t="inlineStr">
+      <c r="D37" s="12">
+        <f>B37*Команда!$B$24/$B$6</f>
+        <v/>
+      </c>
+      <c r="E37" s="12">
+        <f>B37*Команда!$B$24/$B$6</f>
+        <v/>
+      </c>
+      <c r="F37" s="7" t="inlineStr">
         <is>
           <t>Переключатель «в себестоимость / из вознаграждения» — на листе «Команда»</t>
         </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="5" t="inlineStr">
-        <is>
-          <t>СЕБЕСТОИМОСТЬ НА ГОСТЯ</t>
-        </is>
-      </c>
-      <c r="D37" s="13">
-        <f>SUM(D15:D36)</f>
-        <v/>
-      </c>
-      <c r="E37" s="13">
-        <f>SUM(E15:E36)</f>
-        <v/>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="5" t="inlineStr">
         <is>
+          <t>СЕБЕСТОИМОСТЬ НА ГОСТЯ</t>
+        </is>
+      </c>
+      <c r="D38" s="13">
+        <f>SUM(D15:D37)</f>
+        <v/>
+      </c>
+      <c r="E38" s="13">
+        <f>SUM(E15:E37)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="5" t="inlineStr">
+        <is>
           <t>Вознаграждение La Royal</t>
         </is>
       </c>
-      <c r="D38" s="12">
-        <f>D37*$B$11</f>
-        <v/>
-      </c>
-      <c r="E38" s="12">
-        <f>E37*$B$11</f>
-        <v/>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="14" t="inlineStr">
+      <c r="D39" s="12">
+        <f>D38*$B$11</f>
+        <v/>
+      </c>
+      <c r="E39" s="12">
+        <f>E38*$B$11</f>
+        <v/>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="14" t="inlineStr">
         <is>
           <t>ЦЕНА ДЛЯ ГОСТЯ</t>
         </is>
       </c>
-      <c r="D39" s="15">
-        <f>D37+D38</f>
-        <v/>
-      </c>
-      <c r="E39" s="15">
-        <f>E37+E38</f>
-        <v/>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="2" t="inlineStr">
-        <is>
-          <t>Вознаграждение со всей группы</t>
-        </is>
-      </c>
-      <c r="D40" s="16">
-        <f>D38*$B$6-Команда!$B$22*(1-Команда!$B$24)</f>
-        <v/>
-      </c>
-      <c r="E40" s="16">
-        <f>E38*$B$6-Команда!$B$22*(1-Команда!$B$24)</f>
-        <v/>
-      </c>
-      <c r="F40" s="2" t="inlineStr">
-        <is>
-          <t>Если команда идёт из вознаграждения, её расходы вычитаются здесь</t>
-        </is>
+      <c r="D40" s="15">
+        <f>D38+D39</f>
+        <v/>
+      </c>
+      <c r="E40" s="15">
+        <f>E38+E39</f>
+        <v/>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>Если 15 % считать долей в цене, а не наценкой</t>
-        </is>
-      </c>
-      <c r="D41" s="17">
-        <f>D37/(1-$B$11)</f>
-        <v/>
-      </c>
-      <c r="E41" s="17">
-        <f>E37/(1-$B$11)</f>
-        <v/>
+          <t>Вознаграждение со всей группы</t>
+        </is>
+      </c>
+      <c r="D41" s="16">
+        <f>D39*$B$6-Команда!$B$22*(1-Команда!$B$24)</f>
+        <v/>
+      </c>
+      <c r="E41" s="16">
+        <f>E39*$B$6-Команда!$B$22*(1-Команда!$B$24)</f>
+        <v/>
+      </c>
+      <c r="F41" s="2" t="inlineStr">
+        <is>
+          <t>Если команда идёт из вознаграждения, её расходы вычитаются здесь</t>
+        </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
+          <t>Если 15 % считать долей в цене, а не наценкой</t>
+        </is>
+      </c>
+      <c r="D42" s="17">
+        <f>D38/(1-$B$11)</f>
+        <v/>
+      </c>
+      <c r="E42" s="17">
+        <f>E38/(1-$B$11)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="2" t="inlineStr">
+        <is>
           <t>Разница между двумя трактовками, на гостя</t>
         </is>
       </c>
-      <c r="D42" s="17">
-        <f>D41-D39</f>
-        <v/>
-      </c>
-      <c r="E42" s="17">
-        <f>E41-E39</f>
-        <v/>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" s="18" t="inlineStr">
+      <c r="D43" s="17">
+        <f>D42-D40</f>
+        <v/>
+      </c>
+      <c r="E43" s="17">
+        <f>E42-E40</f>
+        <v/>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="18" t="inlineStr">
         <is>
           <t>Пока в столбце «Что уточнить» есть розовые строки, итог занижен и клиенту не называется.</t>
         </is>
@@ -1749,12 +1777,12 @@
         </is>
       </c>
       <c r="B19" s="12">
-        <f>$B$7*760</f>
+        <f>$B$7*760+$B$7*360</f>
         <v/>
       </c>
       <c r="D19" s="7" t="inlineStr">
         <is>
-          <t>150+150+90+120+250 на человека</t>
+          <t>рестораны 760 + билеты в Гизу 360</t>
         </is>
       </c>
     </row>

</xml_diff>